<commit_message>
template-form.xlsx: G/H 현금가 빈칸 처리 + IFERROR 자동계산
- 54행 모두 G(번이 현금가)/H(기변 현금가) 빈칸 — 매장이 직접 입력
- I/J 봉이지원금 자동계산을 IFERROR로 래핑 (빈 행은 빈칸 표시)
- footer 안내 보강

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template-form.xlsx
+++ b/docs/template-form.xlsx
@@ -1292,18 +1292,14 @@
       <c r="F3" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G3" s="46" t="n">
-        <v>-10</v>
-      </c>
-      <c r="H3" s="46" t="n">
-        <v>5</v>
-      </c>
+      <c r="G3" s="46" t="n"/>
+      <c r="H3" s="46" t="n"/>
       <c r="I3" s="47">
-        <f>D3-F3-G3</f>
+        <f>IFERROR(D3-F3-G3,"")</f>
         <v/>
       </c>
       <c r="J3" s="47">
-        <f>D3-F3-H3</f>
+        <f>IFERROR(D3-F3-H3,"")</f>
         <v/>
       </c>
     </row>
@@ -1334,18 +1330,14 @@
       <c r="F4" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G4" s="46" t="n">
-        <v>9</v>
-      </c>
-      <c r="H4" s="46" t="n">
-        <v>34</v>
-      </c>
+      <c r="G4" s="46" t="n"/>
+      <c r="H4" s="46" t="n"/>
       <c r="I4" s="47">
-        <f>D4-F4-G4</f>
+        <f>IFERROR(D4-F4-G4,"")</f>
         <v/>
       </c>
       <c r="J4" s="47">
-        <f>D4-F4-H4</f>
+        <f>IFERROR(D4-F4-H4,"")</f>
         <v/>
       </c>
     </row>
@@ -1376,18 +1368,14 @@
       <c r="F5" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G5" s="46" t="n">
-        <v>44</v>
-      </c>
-      <c r="H5" s="46" t="n">
-        <v>64</v>
-      </c>
+      <c r="G5" s="46" t="n"/>
+      <c r="H5" s="46" t="n"/>
       <c r="I5" s="47">
-        <f>D5-F5-G5</f>
+        <f>IFERROR(D5-F5-G5,"")</f>
         <v/>
       </c>
       <c r="J5" s="47">
-        <f>D5-F5-H5</f>
+        <f>IFERROR(D5-F5-H5,"")</f>
         <v/>
       </c>
     </row>
@@ -1418,18 +1406,14 @@
       <c r="F6" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G6" s="46" t="n">
-        <v>19</v>
-      </c>
-      <c r="H6" s="46" t="n">
-        <v>44</v>
-      </c>
+      <c r="G6" s="46" t="n"/>
+      <c r="H6" s="46" t="n"/>
       <c r="I6" s="47">
-        <f>D6-F6-G6</f>
+        <f>IFERROR(D6-F6-G6,"")</f>
         <v/>
       </c>
       <c r="J6" s="47">
-        <f>D6-F6-H6</f>
+        <f>IFERROR(D6-F6-H6,"")</f>
         <v/>
       </c>
     </row>
@@ -1460,18 +1444,14 @@
       <c r="F7" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G7" s="46" t="n">
-        <v>127</v>
-      </c>
-      <c r="H7" s="46" t="n">
-        <v>139</v>
-      </c>
+      <c r="G7" s="46" t="n"/>
+      <c r="H7" s="46" t="n"/>
       <c r="I7" s="47">
-        <f>D7-F7-G7</f>
+        <f>IFERROR(D7-F7-G7,"")</f>
         <v/>
       </c>
       <c r="J7" s="47">
-        <f>D7-F7-H7</f>
+        <f>IFERROR(D7-F7-H7,"")</f>
         <v/>
       </c>
     </row>
@@ -1502,18 +1482,14 @@
       <c r="F8" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G8" s="46" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="46" t="n">
-        <v>59</v>
-      </c>
+      <c r="G8" s="46" t="n"/>
+      <c r="H8" s="46" t="n"/>
       <c r="I8" s="47">
-        <f>D8-F8-G8</f>
+        <f>IFERROR(D8-F8-G8,"")</f>
         <v/>
       </c>
       <c r="J8" s="47">
-        <f>D8-F8-H8</f>
+        <f>IFERROR(D8-F8-H8,"")</f>
         <v/>
       </c>
     </row>
@@ -1544,18 +1520,14 @@
       <c r="F9" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G9" s="46" t="n">
-        <v>25</v>
-      </c>
-      <c r="H9" s="46" t="n">
-        <v>79</v>
-      </c>
+      <c r="G9" s="46" t="n"/>
+      <c r="H9" s="46" t="n"/>
       <c r="I9" s="47">
-        <f>D9-F9-G9</f>
+        <f>IFERROR(D9-F9-G9,"")</f>
         <v/>
       </c>
       <c r="J9" s="47">
-        <f>D9-F9-H9</f>
+        <f>IFERROR(D9-F9-H9,"")</f>
         <v/>
       </c>
     </row>
@@ -1586,18 +1558,14 @@
       <c r="F10" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G10" s="46" t="n">
-        <v>59</v>
-      </c>
-      <c r="H10" s="46" t="n">
-        <v>114</v>
-      </c>
+      <c r="G10" s="46" t="n"/>
+      <c r="H10" s="46" t="n"/>
       <c r="I10" s="47">
-        <f>D10-F10-G10</f>
+        <f>IFERROR(D10-F10-G10,"")</f>
         <v/>
       </c>
       <c r="J10" s="47">
-        <f>D10-F10-H10</f>
+        <f>IFERROR(D10-F10-H10,"")</f>
         <v/>
       </c>
     </row>
@@ -1628,18 +1596,14 @@
       <c r="F11" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G11" s="46" t="n">
-        <v>39</v>
-      </c>
-      <c r="H11" s="46" t="n">
-        <v>37</v>
-      </c>
+      <c r="G11" s="46" t="n"/>
+      <c r="H11" s="46" t="n"/>
       <c r="I11" s="47">
-        <f>D11-F11-G11</f>
+        <f>IFERROR(D11-F11-G11,"")</f>
         <v/>
       </c>
       <c r="J11" s="47">
-        <f>D11-F11-H11</f>
+        <f>IFERROR(D11-F11-H11,"")</f>
         <v/>
       </c>
     </row>
@@ -1670,18 +1634,14 @@
       <c r="F12" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G12" s="46" t="n">
-        <v>-35</v>
-      </c>
-      <c r="H12" s="46" t="n">
-        <v>-5</v>
-      </c>
+      <c r="G12" s="46" t="n"/>
+      <c r="H12" s="46" t="n"/>
       <c r="I12" s="47">
-        <f>D12-F12-G12</f>
+        <f>IFERROR(D12-F12-G12,"")</f>
         <v/>
       </c>
       <c r="J12" s="47">
-        <f>D12-F12-H12</f>
+        <f>IFERROR(D12-F12-H12,"")</f>
         <v/>
       </c>
     </row>
@@ -1712,18 +1672,14 @@
       <c r="F13" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G13" s="46" t="n">
-        <v>19</v>
-      </c>
-      <c r="H13" s="46" t="n">
-        <v>59</v>
-      </c>
+      <c r="G13" s="46" t="n"/>
+      <c r="H13" s="46" t="n"/>
       <c r="I13" s="47">
-        <f>D13-F13-G13</f>
+        <f>IFERROR(D13-F13-G13,"")</f>
         <v/>
       </c>
       <c r="J13" s="47">
-        <f>D13-F13-H13</f>
+        <f>IFERROR(D13-F13-H13,"")</f>
         <v/>
       </c>
     </row>
@@ -1754,18 +1710,14 @@
       <c r="F14" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G14" s="46" t="n">
-        <v>74</v>
-      </c>
-      <c r="H14" s="46" t="n">
-        <v>79</v>
-      </c>
+      <c r="G14" s="46" t="n"/>
+      <c r="H14" s="46" t="n"/>
       <c r="I14" s="47">
-        <f>D14-F14-G14</f>
+        <f>IFERROR(D14-F14-G14,"")</f>
         <v/>
       </c>
       <c r="J14" s="47">
-        <f>D14-F14-H14</f>
+        <f>IFERROR(D14-F14-H14,"")</f>
         <v/>
       </c>
     </row>
@@ -1796,18 +1748,14 @@
       <c r="F15" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G15" s="46" t="n">
-        <v>49</v>
-      </c>
-      <c r="H15" s="46" t="n">
-        <v>79</v>
-      </c>
+      <c r="G15" s="46" t="n"/>
+      <c r="H15" s="46" t="n"/>
       <c r="I15" s="47">
-        <f>D15-F15-G15</f>
+        <f>IFERROR(D15-F15-G15,"")</f>
         <v/>
       </c>
       <c r="J15" s="47">
-        <f>D15-F15-H15</f>
+        <f>IFERROR(D15-F15-H15,"")</f>
         <v/>
       </c>
     </row>
@@ -1838,18 +1786,14 @@
       <c r="F16" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G16" s="46" t="n">
-        <v>124</v>
-      </c>
-      <c r="H16" s="46" t="n">
-        <v>129</v>
-      </c>
+      <c r="G16" s="46" t="n"/>
+      <c r="H16" s="46" t="n"/>
       <c r="I16" s="47">
-        <f>D16-F16-G16</f>
+        <f>IFERROR(D16-F16-G16,"")</f>
         <v/>
       </c>
       <c r="J16" s="47">
-        <f>D16-F16-H16</f>
+        <f>IFERROR(D16-F16-H16,"")</f>
         <v/>
       </c>
     </row>
@@ -1880,18 +1824,14 @@
       <c r="F17" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G17" s="46" t="n">
-        <v>9</v>
-      </c>
-      <c r="H17" s="46" t="n">
-        <v>54</v>
-      </c>
+      <c r="G17" s="46" t="n"/>
+      <c r="H17" s="46" t="n"/>
       <c r="I17" s="47">
-        <f>D17-F17-G17</f>
+        <f>IFERROR(D17-F17-G17,"")</f>
         <v/>
       </c>
       <c r="J17" s="47">
-        <f>D17-F17-H17</f>
+        <f>IFERROR(D17-F17-H17,"")</f>
         <v/>
       </c>
     </row>
@@ -1922,18 +1862,14 @@
       <c r="F18" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G18" s="46" t="n">
-        <v>49</v>
-      </c>
-      <c r="H18" s="46" t="n">
-        <v>84</v>
-      </c>
+      <c r="G18" s="46" t="n"/>
+      <c r="H18" s="46" t="n"/>
       <c r="I18" s="47">
-        <f>D18-F18-G18</f>
+        <f>IFERROR(D18-F18-G18,"")</f>
         <v/>
       </c>
       <c r="J18" s="47">
-        <f>D18-F18-H18</f>
+        <f>IFERROR(D18-F18-H18,"")</f>
         <v/>
       </c>
     </row>
@@ -1964,18 +1900,14 @@
       <c r="F19" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G19" s="46" t="n">
-        <v>59</v>
-      </c>
-      <c r="H19" s="46" t="n">
-        <v>104</v>
-      </c>
+      <c r="G19" s="46" t="n"/>
+      <c r="H19" s="46" t="n"/>
       <c r="I19" s="47">
-        <f>D19-F19-G19</f>
+        <f>IFERROR(D19-F19-G19,"")</f>
         <v/>
       </c>
       <c r="J19" s="47">
-        <f>D19-F19-H19</f>
+        <f>IFERROR(D19-F19-H19,"")</f>
         <v/>
       </c>
     </row>
@@ -2006,18 +1938,14 @@
       <c r="F20" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="G20" s="46" t="n">
-        <v>109</v>
-      </c>
-      <c r="H20" s="46" t="n">
-        <v>144</v>
-      </c>
+      <c r="G20" s="46" t="n"/>
+      <c r="H20" s="46" t="n"/>
       <c r="I20" s="47">
-        <f>D20-F20-G20</f>
+        <f>IFERROR(D20-F20-G20,"")</f>
         <v/>
       </c>
       <c r="J20" s="47">
-        <f>D20-F20-H20</f>
+        <f>IFERROR(D20-F20-H20,"")</f>
         <v/>
       </c>
     </row>
@@ -2048,18 +1976,14 @@
       <c r="F21" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G21" s="46" t="n">
-        <v>-20</v>
-      </c>
-      <c r="H21" s="46" t="n">
-        <v>-15</v>
-      </c>
+      <c r="G21" s="46" t="n"/>
+      <c r="H21" s="46" t="n"/>
       <c r="I21" s="47">
-        <f>D21-F21-G21</f>
+        <f>IFERROR(D21-F21-G21,"")</f>
         <v/>
       </c>
       <c r="J21" s="47">
-        <f>D21-F21-H21</f>
+        <f>IFERROR(D21-F21-H21,"")</f>
         <v/>
       </c>
     </row>
@@ -2090,18 +2014,14 @@
       <c r="F22" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G22" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="46" t="n">
-        <v>5</v>
-      </c>
+      <c r="G22" s="46" t="n"/>
+      <c r="H22" s="46" t="n"/>
       <c r="I22" s="47">
-        <f>D22-F22-G22</f>
+        <f>IFERROR(D22-F22-G22,"")</f>
         <v/>
       </c>
       <c r="J22" s="47">
-        <f>D22-F22-H22</f>
+        <f>IFERROR(D22-F22-H22,"")</f>
         <v/>
       </c>
     </row>
@@ -2132,18 +2052,14 @@
       <c r="F23" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G23" s="46" t="n">
-        <v>34</v>
-      </c>
-      <c r="H23" s="46" t="n">
-        <v>39</v>
-      </c>
+      <c r="G23" s="46" t="n"/>
+      <c r="H23" s="46" t="n"/>
       <c r="I23" s="47">
-        <f>D23-F23-G23</f>
+        <f>IFERROR(D23-F23-G23,"")</f>
         <v/>
       </c>
       <c r="J23" s="47">
-        <f>D23-F23-H23</f>
+        <f>IFERROR(D23-F23-H23,"")</f>
         <v/>
       </c>
     </row>
@@ -2174,18 +2090,14 @@
       <c r="F24" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G24" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="46" t="n">
-        <v>5</v>
-      </c>
+      <c r="G24" s="46" t="n"/>
+      <c r="H24" s="46" t="n"/>
       <c r="I24" s="47">
-        <f>D24-F24-G24</f>
+        <f>IFERROR(D24-F24-G24,"")</f>
         <v/>
       </c>
       <c r="J24" s="47">
-        <f>D24-F24-H24</f>
+        <f>IFERROR(D24-F24-H24,"")</f>
         <v/>
       </c>
     </row>
@@ -2216,18 +2128,14 @@
       <c r="F25" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G25" s="46" t="n">
-        <v>99</v>
-      </c>
-      <c r="H25" s="46" t="n">
-        <v>104</v>
-      </c>
+      <c r="G25" s="46" t="n"/>
+      <c r="H25" s="46" t="n"/>
       <c r="I25" s="47">
-        <f>D25-F25-G25</f>
+        <f>IFERROR(D25-F25-G25,"")</f>
         <v/>
       </c>
       <c r="J25" s="47">
-        <f>D25-F25-H25</f>
+        <f>IFERROR(D25-F25-H25,"")</f>
         <v/>
       </c>
     </row>
@@ -2258,18 +2166,14 @@
       <c r="F26" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G26" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="46" t="n">
-        <v>19</v>
-      </c>
+      <c r="G26" s="46" t="n"/>
+      <c r="H26" s="46" t="n"/>
       <c r="I26" s="47">
-        <f>D26-F26-G26</f>
+        <f>IFERROR(D26-F26-G26,"")</f>
         <v/>
       </c>
       <c r="J26" s="47">
-        <f>D26-F26-H26</f>
+        <f>IFERROR(D26-F26-H26,"")</f>
         <v/>
       </c>
     </row>
@@ -2300,18 +2204,14 @@
       <c r="F27" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G27" s="46" t="n">
-        <v>19</v>
-      </c>
-      <c r="H27" s="46" t="n">
-        <v>39</v>
-      </c>
+      <c r="G27" s="46" t="n"/>
+      <c r="H27" s="46" t="n"/>
       <c r="I27" s="47">
-        <f>D27-F27-G27</f>
+        <f>IFERROR(D27-F27-G27,"")</f>
         <v/>
       </c>
       <c r="J27" s="47">
-        <f>D27-F27-H27</f>
+        <f>IFERROR(D27-F27-H27,"")</f>
         <v/>
       </c>
     </row>
@@ -2342,18 +2242,14 @@
       <c r="F28" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G28" s="46" t="n">
-        <v>54</v>
-      </c>
-      <c r="H28" s="46" t="n">
-        <v>74</v>
-      </c>
+      <c r="G28" s="46" t="n"/>
+      <c r="H28" s="46" t="n"/>
       <c r="I28" s="47">
-        <f>D28-F28-G28</f>
+        <f>IFERROR(D28-F28-G28,"")</f>
         <v/>
       </c>
       <c r="J28" s="47">
-        <f>D28-F28-H28</f>
+        <f>IFERROR(D28-F28-H28,"")</f>
         <v/>
       </c>
     </row>
@@ -2384,18 +2280,14 @@
       <c r="F29" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G29" s="46" t="n">
-        <v>5</v>
-      </c>
-      <c r="H29" s="46" t="n">
-        <v>0</v>
-      </c>
+      <c r="G29" s="46" t="n"/>
+      <c r="H29" s="46" t="n"/>
       <c r="I29" s="47">
-        <f>D29-F29-G29</f>
+        <f>IFERROR(D29-F29-G29,"")</f>
         <v/>
       </c>
       <c r="J29" s="47">
-        <f>D29-F29-H29</f>
+        <f>IFERROR(D29-F29-H29,"")</f>
         <v/>
       </c>
     </row>
@@ -2426,18 +2318,14 @@
       <c r="F30" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G30" s="46" t="n">
-        <v>-40</v>
-      </c>
-      <c r="H30" s="46" t="n">
-        <v>-25</v>
-      </c>
+      <c r="G30" s="46" t="n"/>
+      <c r="H30" s="46" t="n"/>
       <c r="I30" s="47">
-        <f>D30-F30-G30</f>
+        <f>IFERROR(D30-F30-G30,"")</f>
         <v/>
       </c>
       <c r="J30" s="47">
-        <f>D30-F30-H30</f>
+        <f>IFERROR(D30-F30-H30,"")</f>
         <v/>
       </c>
     </row>
@@ -2468,18 +2356,14 @@
       <c r="F31" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G31" s="46" t="n">
-        <v>-55</v>
-      </c>
-      <c r="H31" s="46" t="n">
-        <v>-30</v>
-      </c>
+      <c r="G31" s="46" t="n"/>
+      <c r="H31" s="46" t="n"/>
       <c r="I31" s="47">
-        <f>D31-F31-G31</f>
+        <f>IFERROR(D31-F31-G31,"")</f>
         <v/>
       </c>
       <c r="J31" s="47">
-        <f>D31-F31-H31</f>
+        <f>IFERROR(D31-F31-H31,"")</f>
         <v/>
       </c>
     </row>
@@ -2510,18 +2394,14 @@
       <c r="F32" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G32" s="46" t="n">
-        <v>-45</v>
-      </c>
-      <c r="H32" s="46" t="n">
-        <v>-20</v>
-      </c>
+      <c r="G32" s="46" t="n"/>
+      <c r="H32" s="46" t="n"/>
       <c r="I32" s="47">
-        <f>D32-F32-G32</f>
+        <f>IFERROR(D32-F32-G32,"")</f>
         <v/>
       </c>
       <c r="J32" s="47">
-        <f>D32-F32-H32</f>
+        <f>IFERROR(D32-F32-H32,"")</f>
         <v/>
       </c>
     </row>
@@ -2552,18 +2432,14 @@
       <c r="F33" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G33" s="46" t="n">
-        <v>-25</v>
-      </c>
-      <c r="H33" s="46" t="n">
-        <v>0</v>
-      </c>
+      <c r="G33" s="46" t="n"/>
+      <c r="H33" s="46" t="n"/>
       <c r="I33" s="47">
-        <f>D33-F33-G33</f>
+        <f>IFERROR(D33-F33-G33,"")</f>
         <v/>
       </c>
       <c r="J33" s="47">
-        <f>D33-F33-H33</f>
+        <f>IFERROR(D33-F33-H33,"")</f>
         <v/>
       </c>
     </row>
@@ -2594,18 +2470,14 @@
       <c r="F34" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G34" s="46" t="n">
-        <v>9</v>
-      </c>
-      <c r="H34" s="46" t="n">
-        <v>34</v>
-      </c>
+      <c r="G34" s="46" t="n"/>
+      <c r="H34" s="46" t="n"/>
       <c r="I34" s="47">
-        <f>D34-F34-G34</f>
+        <f>IFERROR(D34-F34-G34,"")</f>
         <v/>
       </c>
       <c r="J34" s="47">
-        <f>D34-F34-H34</f>
+        <f>IFERROR(D34-F34-H34,"")</f>
         <v/>
       </c>
     </row>
@@ -2636,18 +2508,14 @@
       <c r="F35" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G35" s="46" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H35" s="46" t="n">
-        <v>24</v>
-      </c>
+      <c r="G35" s="46" t="n"/>
+      <c r="H35" s="46" t="n"/>
       <c r="I35" s="47">
-        <f>D35-F35-G35</f>
+        <f>IFERROR(D35-F35-G35,"")</f>
         <v/>
       </c>
       <c r="J35" s="47">
-        <f>D35-F35-H35</f>
+        <f>IFERROR(D35-F35-H35,"")</f>
         <v/>
       </c>
     </row>
@@ -2678,18 +2546,14 @@
       <c r="F36" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G36" s="46" t="n">
-        <v>34</v>
-      </c>
-      <c r="H36" s="46" t="n">
-        <v>54</v>
-      </c>
+      <c r="G36" s="46" t="n"/>
+      <c r="H36" s="46" t="n"/>
       <c r="I36" s="47">
-        <f>D36-F36-G36</f>
+        <f>IFERROR(D36-F36-G36,"")</f>
         <v/>
       </c>
       <c r="J36" s="47">
-        <f>D36-F36-H36</f>
+        <f>IFERROR(D36-F36-H36,"")</f>
         <v/>
       </c>
     </row>
@@ -2720,18 +2584,14 @@
       <c r="F37" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G37" s="46" t="n">
-        <v>59</v>
-      </c>
-      <c r="H37" s="46" t="n">
-        <v>79</v>
-      </c>
+      <c r="G37" s="46" t="n"/>
+      <c r="H37" s="46" t="n"/>
       <c r="I37" s="47">
-        <f>D37-F37-G37</f>
+        <f>IFERROR(D37-F37-G37,"")</f>
         <v/>
       </c>
       <c r="J37" s="47">
-        <f>D37-F37-H37</f>
+        <f>IFERROR(D37-F37-H37,"")</f>
         <v/>
       </c>
     </row>
@@ -2762,18 +2622,14 @@
       <c r="F38" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="G38" s="46" t="n">
-        <v>94</v>
-      </c>
-      <c r="H38" s="46" t="n">
-        <v>124</v>
-      </c>
+      <c r="G38" s="46" t="n"/>
+      <c r="H38" s="46" t="n"/>
       <c r="I38" s="47">
-        <f>D38-F38-G38</f>
+        <f>IFERROR(D38-F38-G38,"")</f>
         <v/>
       </c>
       <c r="J38" s="47">
-        <f>D38-F38-H38</f>
+        <f>IFERROR(D38-F38-H38,"")</f>
         <v/>
       </c>
     </row>
@@ -2804,18 +2660,14 @@
       <c r="F39" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G39" s="46" t="n">
-        <v>-25</v>
-      </c>
-      <c r="H39" s="46" t="n">
-        <v>-20</v>
-      </c>
+      <c r="G39" s="46" t="n"/>
+      <c r="H39" s="46" t="n"/>
       <c r="I39" s="47">
-        <f>D39-F39-G39</f>
+        <f>IFERROR(D39-F39-G39,"")</f>
         <v/>
       </c>
       <c r="J39" s="47">
-        <f>D39-F39-H39</f>
+        <f>IFERROR(D39-F39-H39,"")</f>
         <v/>
       </c>
     </row>
@@ -2846,18 +2698,14 @@
       <c r="F40" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G40" s="46" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H40" s="46" t="n">
-        <v>0</v>
-      </c>
+      <c r="G40" s="46" t="n"/>
+      <c r="H40" s="46" t="n"/>
       <c r="I40" s="47">
-        <f>D40-F40-G40</f>
+        <f>IFERROR(D40-F40-G40,"")</f>
         <v/>
       </c>
       <c r="J40" s="47">
-        <f>D40-F40-H40</f>
+        <f>IFERROR(D40-F40-H40,"")</f>
         <v/>
       </c>
     </row>
@@ -2888,18 +2736,14 @@
       <c r="F41" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G41" s="46" t="n">
-        <v>29</v>
-      </c>
-      <c r="H41" s="46" t="n">
-        <v>34</v>
-      </c>
+      <c r="G41" s="46" t="n"/>
+      <c r="H41" s="46" t="n"/>
       <c r="I41" s="47">
-        <f>D41-F41-G41</f>
+        <f>IFERROR(D41-F41-G41,"")</f>
         <v/>
       </c>
       <c r="J41" s="47">
-        <f>D41-F41-H41</f>
+        <f>IFERROR(D41-F41-H41,"")</f>
         <v/>
       </c>
     </row>
@@ -2930,18 +2774,14 @@
       <c r="F42" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G42" s="46" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H42" s="46" t="n">
-        <v>-5</v>
-      </c>
+      <c r="G42" s="46" t="n"/>
+      <c r="H42" s="46" t="n"/>
       <c r="I42" s="47">
-        <f>D42-F42-G42</f>
+        <f>IFERROR(D42-F42-G42,"")</f>
         <v/>
       </c>
       <c r="J42" s="47">
-        <f>D42-F42-H42</f>
+        <f>IFERROR(D42-F42-H42,"")</f>
         <v/>
       </c>
     </row>
@@ -2972,18 +2812,14 @@
       <c r="F43" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G43" s="46" t="n">
-        <v>94</v>
-      </c>
-      <c r="H43" s="46" t="n">
-        <v>94</v>
-      </c>
+      <c r="G43" s="46" t="n"/>
+      <c r="H43" s="46" t="n"/>
       <c r="I43" s="47">
-        <f>D43-F43-G43</f>
+        <f>IFERROR(D43-F43-G43,"")</f>
         <v/>
       </c>
       <c r="J43" s="47">
-        <f>D43-F43-H43</f>
+        <f>IFERROR(D43-F43-H43,"")</f>
         <v/>
       </c>
     </row>
@@ -3014,18 +2850,14 @@
       <c r="F44" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G44" s="46" t="n">
-        <v>19</v>
-      </c>
-      <c r="H44" s="46" t="n">
-        <v>24</v>
-      </c>
+      <c r="G44" s="46" t="n"/>
+      <c r="H44" s="46" t="n"/>
       <c r="I44" s="47">
-        <f>D44-F44-G44</f>
+        <f>IFERROR(D44-F44-G44,"")</f>
         <v/>
       </c>
       <c r="J44" s="47">
-        <f>D44-F44-H44</f>
+        <f>IFERROR(D44-F44-H44,"")</f>
         <v/>
       </c>
     </row>
@@ -3056,18 +2888,14 @@
       <c r="F45" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G45" s="46" t="n">
-        <v>39</v>
-      </c>
-      <c r="H45" s="46" t="n">
-        <v>44</v>
-      </c>
+      <c r="G45" s="46" t="n"/>
+      <c r="H45" s="46" t="n"/>
       <c r="I45" s="47">
-        <f>D45-F45-G45</f>
+        <f>IFERROR(D45-F45-G45,"")</f>
         <v/>
       </c>
       <c r="J45" s="47">
-        <f>D45-F45-H45</f>
+        <f>IFERROR(D45-F45-H45,"")</f>
         <v/>
       </c>
     </row>
@@ -3098,18 +2926,14 @@
       <c r="F46" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G46" s="46" t="n">
-        <v>74</v>
-      </c>
-      <c r="H46" s="46" t="n">
-        <v>78</v>
-      </c>
+      <c r="G46" s="46" t="n"/>
+      <c r="H46" s="46" t="n"/>
       <c r="I46" s="47">
-        <f>D46-F46-G46</f>
+        <f>IFERROR(D46-F46-G46,"")</f>
         <v/>
       </c>
       <c r="J46" s="47">
-        <f>D46-F46-H46</f>
+        <f>IFERROR(D46-F46-H46,"")</f>
         <v/>
       </c>
     </row>
@@ -3140,18 +2964,14 @@
       <c r="F47" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G47" s="46" t="n">
-        <v>-20</v>
-      </c>
-      <c r="H47" s="46" t="n">
-        <v>5</v>
-      </c>
+      <c r="G47" s="46" t="n"/>
+      <c r="H47" s="46" t="n"/>
       <c r="I47" s="47">
-        <f>D47-F47-G47</f>
+        <f>IFERROR(D47-F47-G47,"")</f>
         <v/>
       </c>
       <c r="J47" s="47">
-        <f>D47-F47-H47</f>
+        <f>IFERROR(D47-F47-H47,"")</f>
         <v/>
       </c>
     </row>
@@ -3182,18 +3002,14 @@
       <c r="F48" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G48" s="46" t="n">
-        <v>-50</v>
-      </c>
-      <c r="H48" s="46" t="n">
-        <v>-15</v>
-      </c>
+      <c r="G48" s="46" t="n"/>
+      <c r="H48" s="46" t="n"/>
       <c r="I48" s="47">
-        <f>D48-F48-G48</f>
+        <f>IFERROR(D48-F48-G48,"")</f>
         <v/>
       </c>
       <c r="J48" s="47">
-        <f>D48-F48-H48</f>
+        <f>IFERROR(D48-F48-H48,"")</f>
         <v/>
       </c>
     </row>
@@ -3224,18 +3040,14 @@
       <c r="F49" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G49" s="46" t="n">
-        <v>-40</v>
-      </c>
-      <c r="H49" s="46" t="n">
-        <v>14</v>
-      </c>
+      <c r="G49" s="46" t="n"/>
+      <c r="H49" s="46" t="n"/>
       <c r="I49" s="47">
-        <f>D49-F49-G49</f>
+        <f>IFERROR(D49-F49-G49,"")</f>
         <v/>
       </c>
       <c r="J49" s="47">
-        <f>D49-F49-H49</f>
+        <f>IFERROR(D49-F49-H49,"")</f>
         <v/>
       </c>
     </row>
@@ -3266,18 +3078,14 @@
       <c r="F50" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G50" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="46" t="n">
-        <v>54</v>
-      </c>
+      <c r="G50" s="46" t="n"/>
+      <c r="H50" s="46" t="n"/>
       <c r="I50" s="47">
-        <f>D50-F50-G50</f>
+        <f>IFERROR(D50-F50-G50,"")</f>
         <v/>
       </c>
       <c r="J50" s="47">
-        <f>D50-F50-H50</f>
+        <f>IFERROR(D50-F50-H50,"")</f>
         <v/>
       </c>
     </row>
@@ -3308,18 +3116,14 @@
       <c r="F51" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G51" s="46" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H51" s="46" t="n">
-        <v>44</v>
-      </c>
+      <c r="G51" s="46" t="n"/>
+      <c r="H51" s="46" t="n"/>
       <c r="I51" s="47">
-        <f>D51-F51-G51</f>
+        <f>IFERROR(D51-F51-G51,"")</f>
         <v/>
       </c>
       <c r="J51" s="47">
-        <f>D51-F51-H51</f>
+        <f>IFERROR(D51-F51-H51,"")</f>
         <v/>
       </c>
     </row>
@@ -3350,18 +3154,14 @@
       <c r="F52" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G52" s="46" t="n">
-        <v>29</v>
-      </c>
-      <c r="H52" s="46" t="n">
-        <v>84</v>
-      </c>
+      <c r="G52" s="46" t="n"/>
+      <c r="H52" s="46" t="n"/>
       <c r="I52" s="47">
-        <f>D52-F52-G52</f>
+        <f>IFERROR(D52-F52-G52,"")</f>
         <v/>
       </c>
       <c r="J52" s="47">
-        <f>D52-F52-H52</f>
+        <f>IFERROR(D52-F52-H52,"")</f>
         <v/>
       </c>
     </row>
@@ -3392,18 +3192,14 @@
       <c r="F53" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G53" s="46" t="n">
-        <v>-15</v>
-      </c>
-      <c r="H53" s="46" t="n">
-        <v>19</v>
-      </c>
+      <c r="G53" s="46" t="n"/>
+      <c r="H53" s="46" t="n"/>
       <c r="I53" s="47">
-        <f>D53-F53-G53</f>
+        <f>IFERROR(D53-F53-G53,"")</f>
         <v/>
       </c>
       <c r="J53" s="47">
-        <f>D53-F53-H53</f>
+        <f>IFERROR(D53-F53-H53,"")</f>
         <v/>
       </c>
     </row>
@@ -3434,18 +3230,14 @@
       <c r="F54" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G54" s="46" t="n">
-        <v>-40</v>
-      </c>
-      <c r="H54" s="46" t="n">
-        <v>49</v>
-      </c>
+      <c r="G54" s="46" t="n"/>
+      <c r="H54" s="46" t="n"/>
       <c r="I54" s="47">
-        <f>D54-F54-G54</f>
+        <f>IFERROR(D54-F54-G54,"")</f>
         <v/>
       </c>
       <c r="J54" s="47">
-        <f>D54-F54-H54</f>
+        <f>IFERROR(D54-F54-H54,"")</f>
         <v/>
       </c>
     </row>
@@ -3476,18 +3268,14 @@
       <c r="F55" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G55" s="46" t="n">
-        <v>34</v>
-      </c>
-      <c r="H55" s="46" t="n">
-        <v>69</v>
-      </c>
+      <c r="G55" s="46" t="n"/>
+      <c r="H55" s="46" t="n"/>
       <c r="I55" s="47">
-        <f>D55-F55-G55</f>
+        <f>IFERROR(D55-F55-G55,"")</f>
         <v/>
       </c>
       <c r="J55" s="47">
-        <f>D55-F55-H55</f>
+        <f>IFERROR(D55-F55-H55,"")</f>
         <v/>
       </c>
     </row>
@@ -3518,25 +3306,24 @@
       <c r="F56" s="34" t="n">
         <v>47</v>
       </c>
-      <c r="G56" s="46" t="n">
-        <v>89</v>
-      </c>
-      <c r="H56" s="46" t="n">
-        <v>114</v>
-      </c>
+      <c r="G56" s="46" t="n"/>
+      <c r="H56" s="46" t="n"/>
       <c r="I56" s="47">
-        <f>D56-F56-G56</f>
+        <f>IFERROR(D56-F56-G56,"")</f>
         <v/>
       </c>
       <c r="J56" s="47">
-        <f>D56-F56-H56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="240" customHeight="1">
+        <f>IFERROR(D56-F56-H56,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58" ht="260" customHeight="1">
       <c r="A58" s="38" t="inlineStr">
         <is>
-          <t>※ 입력값: D=출고가, F=공시지원금, G=번이 현금가, H=기변 현금가 (모두 만원 · 음수 허용)
+          <t>※ G(번이 현금가) · H(기변 현금가)는 빈칸 — 매장이 직접 입력
+※ I·J 봉이지원금은 G·H 입력 시 자동 계산 (빈 행은 빈칸 표시)
+※ 입력값: D=출고가, F=공시지원금, G=번이 현금가, H=기변 현금가 (모두 만원 · 음수 허용)
 ※ 자동 계산 (봉이지원금 = 할부 시 페이백 금액 · 역산):
    · I (번이) = D − F − G
    · J (기변) = D − F − H

</xml_diff>

<commit_message>
feat(template): 선약현금가 정적 값 채움 (formula X)
자동계산 로직(formula)은 제거 — 매장이 수정 가능한 정적 숫자로 입력:
- H (번이 선약현금가) = F + G 결과를 plain number로
- J (기변 선약현금가) = F + I 결과를 plain number로

엑셀 수식 (=F2+G2) 사용 X — 단순 숫자라 매장이 직접 덮어쓰기 쉬움.
68셀 정적 값 채움.

샘플:
- SK S26: H=51 J=60
- SK S26U: H=105 J=114
- KT S26: H=60 J=55
- LG S26: H=41 J=43

매장이 공시·선약 매장지원금 차이를 알면 H·J를 직접 수정.
F+G는 기본값으로 제공.

SW v163 → v164

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template-form.xlsx
+++ b/docs/template-form.xlsx
@@ -670,14 +670,14 @@
       <c r="G3">
         <v>-7</v>
       </c>
-      <c r="H3" t="str">
-        <v/>
+      <c r="H3">
+        <v>51</v>
       </c>
       <c r="I3">
         <v>2</v>
       </c>
-      <c r="J3" t="str">
-        <v/>
+      <c r="J3">
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -702,14 +702,14 @@
       <c r="G4">
         <v>13</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
+      <c r="H4">
+        <v>71</v>
       </c>
       <c r="I4">
         <v>22</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
+      <c r="J4">
+        <v>80</v>
       </c>
     </row>
     <row r="5">
@@ -734,14 +734,14 @@
       <c r="G5">
         <v>47</v>
       </c>
-      <c r="H5" t="str">
-        <v/>
+      <c r="H5">
+        <v>105</v>
       </c>
       <c r="I5">
         <v>56</v>
       </c>
-      <c r="J5" t="str">
-        <v/>
+      <c r="J5">
+        <v>114</v>
       </c>
     </row>
     <row r="6">
@@ -766,14 +766,14 @@
       <c r="G6">
         <v>26</v>
       </c>
-      <c r="H6" t="str">
-        <v/>
+      <c r="H6">
+        <v>86</v>
       </c>
       <c r="I6">
         <v>62</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
+      <c r="J6">
+        <v>122</v>
       </c>
     </row>
     <row r="7">
@@ -798,14 +798,14 @@
       <c r="G7">
         <v>133</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
+      <c r="H7">
+        <v>183</v>
       </c>
       <c r="I7">
         <v>156</v>
       </c>
-      <c r="J7" t="str">
-        <v/>
+      <c r="J7">
+        <v>206</v>
       </c>
     </row>
     <row r="8">
@@ -830,14 +830,14 @@
       <c r="G8">
         <v>50</v>
       </c>
-      <c r="H8" t="str">
-        <v/>
+      <c r="H8">
+        <v>110</v>
       </c>
       <c r="I8">
         <v>45</v>
       </c>
-      <c r="J8" t="str">
-        <v/>
+      <c r="J8">
+        <v>105</v>
       </c>
     </row>
     <row r="9">
@@ -862,14 +862,14 @@
       <c r="G9">
         <v>-25</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
+      <c r="H9">
+        <v>25</v>
       </c>
       <c r="I9">
         <v>6</v>
       </c>
-      <c r="J9" t="str">
-        <v/>
+      <c r="J9">
+        <v>56</v>
       </c>
     </row>
     <row r="10">
@@ -894,14 +894,14 @@
       <c r="G10">
         <v>9</v>
       </c>
-      <c r="H10" t="str">
-        <v/>
+      <c r="H10">
+        <v>54</v>
       </c>
       <c r="I10">
         <v>61</v>
       </c>
-      <c r="J10" t="str">
-        <v/>
+      <c r="J10">
+        <v>106</v>
       </c>
     </row>
     <row r="11">
@@ -926,14 +926,14 @@
       <c r="G11">
         <v>47</v>
       </c>
-      <c r="H11" t="str">
-        <v/>
+      <c r="H11">
+        <v>92</v>
       </c>
       <c r="I11">
         <v>89</v>
       </c>
-      <c r="J11" t="str">
-        <v/>
+      <c r="J11">
+        <v>134</v>
       </c>
     </row>
     <row r="12">
@@ -958,14 +958,14 @@
       <c r="G12">
         <v>59</v>
       </c>
-      <c r="H12" t="str">
-        <v/>
+      <c r="H12">
+        <v>104</v>
       </c>
       <c r="I12">
         <v>111</v>
       </c>
-      <c r="J12" t="str">
-        <v/>
+      <c r="J12">
+        <v>156</v>
       </c>
     </row>
     <row r="13">
@@ -990,14 +990,14 @@
       <c r="G13">
         <v>106</v>
       </c>
-      <c r="H13" t="str">
-        <v/>
+      <c r="H13">
+        <v>128</v>
       </c>
       <c r="I13">
         <v>153</v>
       </c>
-      <c r="J13" t="str">
-        <v/>
+      <c r="J13">
+        <v>175</v>
       </c>
     </row>
     <row r="14">
@@ -1022,14 +1022,14 @@
       <c r="G14">
         <v>0</v>
       </c>
-      <c r="H14" t="str">
-        <v/>
+      <c r="H14">
+        <v>60</v>
       </c>
       <c r="I14">
         <v>-5</v>
       </c>
-      <c r="J14" t="str">
-        <v/>
+      <c r="J14">
+        <v>55</v>
       </c>
     </row>
     <row r="15">
@@ -1054,14 +1054,14 @@
       <c r="G15">
         <v>20</v>
       </c>
-      <c r="H15" t="str">
-        <v/>
+      <c r="H15">
+        <v>80</v>
       </c>
       <c r="I15">
         <v>15</v>
       </c>
-      <c r="J15" t="str">
-        <v/>
+      <c r="J15">
+        <v>75</v>
       </c>
     </row>
     <row r="16">
@@ -1086,14 +1086,14 @@
       <c r="G16">
         <v>54</v>
       </c>
-      <c r="H16" t="str">
-        <v/>
+      <c r="H16">
+        <v>114</v>
       </c>
       <c r="I16">
         <v>49</v>
       </c>
-      <c r="J16" t="str">
-        <v/>
+      <c r="J16">
+        <v>109</v>
       </c>
     </row>
     <row r="17">
@@ -1118,14 +1118,14 @@
       <c r="G17">
         <v>15</v>
       </c>
-      <c r="H17" t="str">
-        <v/>
+      <c r="H17">
+        <v>75</v>
       </c>
       <c r="I17">
         <v>32</v>
       </c>
-      <c r="J17" t="str">
-        <v/>
+      <c r="J17">
+        <v>92</v>
       </c>
     </row>
     <row r="18">
@@ -1150,14 +1150,14 @@
       <c r="G18">
         <v>119</v>
       </c>
-      <c r="H18" t="str">
-        <v/>
+      <c r="H18">
+        <v>169</v>
       </c>
       <c r="I18">
         <v>128</v>
       </c>
-      <c r="J18" t="str">
-        <v/>
+      <c r="J18">
+        <v>178</v>
       </c>
     </row>
     <row r="19">
@@ -1182,14 +1182,14 @@
       <c r="G19">
         <v>20</v>
       </c>
-      <c r="H19" t="str">
-        <v/>
+      <c r="H19">
+        <v>80</v>
       </c>
       <c r="I19">
         <v>25</v>
       </c>
-      <c r="J19" t="str">
-        <v/>
+      <c r="J19">
+        <v>85</v>
       </c>
     </row>
     <row r="20">
@@ -1214,14 +1214,14 @@
       <c r="G20">
         <v>-33</v>
       </c>
-      <c r="H20" t="str">
-        <v/>
+      <c r="H20">
+        <v>17</v>
       </c>
       <c r="I20">
         <v>-11</v>
       </c>
-      <c r="J20" t="str">
-        <v/>
+      <c r="J20">
+        <v>39</v>
       </c>
     </row>
     <row r="21">
@@ -1246,14 +1246,14 @@
       <c r="G21">
         <v>12</v>
       </c>
-      <c r="H21" t="str">
-        <v/>
+      <c r="H21">
+        <v>57</v>
       </c>
       <c r="I21">
         <v>45</v>
       </c>
-      <c r="J21" t="str">
-        <v/>
+      <c r="J21">
+        <v>90</v>
       </c>
     </row>
     <row r="22">
@@ -1278,14 +1278,14 @@
       <c r="G22">
         <v>47</v>
       </c>
-      <c r="H22" t="str">
-        <v/>
+      <c r="H22">
+        <v>92</v>
       </c>
       <c r="I22">
         <v>72</v>
       </c>
-      <c r="J22" t="str">
-        <v/>
+      <c r="J22">
+        <v>117</v>
       </c>
     </row>
     <row r="23">
@@ -1310,14 +1310,14 @@
       <c r="G23">
         <v>67</v>
       </c>
-      <c r="H23" t="str">
-        <v/>
+      <c r="H23">
+        <v>112</v>
       </c>
       <c r="I23">
         <v>96</v>
       </c>
-      <c r="J23" t="str">
-        <v/>
+      <c r="J23">
+        <v>141</v>
       </c>
     </row>
     <row r="24">
@@ -1342,14 +1342,14 @@
       <c r="G24">
         <v>111</v>
       </c>
-      <c r="H24" t="str">
-        <v/>
+      <c r="H24">
+        <v>131.1</v>
       </c>
       <c r="I24">
         <v>140</v>
       </c>
-      <c r="J24" t="str">
-        <v/>
+      <c r="J24">
+        <v>160.1</v>
       </c>
     </row>
     <row r="25">
@@ -1374,14 +1374,14 @@
       <c r="G25">
         <v>-29</v>
       </c>
-      <c r="H25" t="str">
-        <v/>
+      <c r="H25">
+        <v>41</v>
       </c>
       <c r="I25">
         <v>-27</v>
       </c>
-      <c r="J25" t="str">
-        <v/>
+      <c r="J25">
+        <v>43</v>
       </c>
     </row>
     <row r="26">
@@ -1406,14 +1406,14 @@
       <c r="G26">
         <v>-9</v>
       </c>
-      <c r="H26" t="str">
-        <v/>
+      <c r="H26">
+        <v>61</v>
       </c>
       <c r="I26">
         <v>-7</v>
       </c>
-      <c r="J26" t="str">
-        <v/>
+      <c r="J26">
+        <v>63</v>
       </c>
     </row>
     <row r="27">
@@ -1438,14 +1438,14 @@
       <c r="G27">
         <v>25</v>
       </c>
-      <c r="H27" t="str">
-        <v/>
+      <c r="H27">
+        <v>95</v>
       </c>
       <c r="I27">
         <v>27</v>
       </c>
-      <c r="J27" t="str">
-        <v/>
+      <c r="J27">
+        <v>97</v>
       </c>
     </row>
     <row r="28">
@@ -1470,14 +1470,14 @@
       <c r="G28">
         <v>15</v>
       </c>
-      <c r="H28" t="str">
-        <v/>
+      <c r="H28">
+        <v>75</v>
       </c>
       <c r="I28">
         <v>4</v>
       </c>
-      <c r="J28" t="str">
-        <v/>
+      <c r="J28">
+        <v>64</v>
       </c>
     </row>
     <row r="29">
@@ -1502,14 +1502,14 @@
       <c r="G29">
         <v>114</v>
       </c>
-      <c r="H29" t="str">
-        <v/>
+      <c r="H29">
+        <v>164</v>
       </c>
       <c r="I29">
         <v>105</v>
       </c>
-      <c r="J29" t="str">
-        <v/>
+      <c r="J29">
+        <v>155</v>
       </c>
     </row>
     <row r="30">
@@ -1534,14 +1534,14 @@
       <c r="G30">
         <v>-6</v>
       </c>
-      <c r="H30" t="str">
-        <v/>
+      <c r="H30">
+        <v>54</v>
       </c>
       <c r="I30">
         <v>15</v>
       </c>
-      <c r="J30" t="str">
-        <v/>
+      <c r="J30">
+        <v>75</v>
       </c>
     </row>
     <row r="31">
@@ -1566,14 +1566,14 @@
       <c r="G31">
         <v>-37</v>
       </c>
-      <c r="H31" t="str">
-        <v/>
+      <c r="H31">
+        <v>13</v>
       </c>
       <c r="I31">
         <v>-4</v>
       </c>
-      <c r="J31" t="str">
-        <v/>
+      <c r="J31">
+        <v>46</v>
       </c>
     </row>
     <row r="32">
@@ -1598,14 +1598,14 @@
       <c r="G32">
         <v>-22</v>
       </c>
-      <c r="H32" t="str">
-        <v/>
+      <c r="H32">
+        <v>23</v>
       </c>
       <c r="I32">
         <v>28</v>
       </c>
-      <c r="J32" t="str">
-        <v/>
+      <c r="J32">
+        <v>73</v>
       </c>
     </row>
     <row r="33">
@@ -1630,14 +1630,14 @@
       <c r="G33">
         <v>-3</v>
       </c>
-      <c r="H33" t="str">
-        <v/>
+      <c r="H33">
+        <v>42</v>
       </c>
       <c r="I33">
         <v>33</v>
       </c>
-      <c r="J33" t="str">
-        <v/>
+      <c r="J33">
+        <v>78</v>
       </c>
     </row>
     <row r="34">
@@ -1662,14 +1662,14 @@
       <c r="G34">
         <v>-28</v>
       </c>
-      <c r="H34" t="str">
-        <v/>
+      <c r="H34">
+        <v>17</v>
       </c>
       <c r="I34">
         <v>63</v>
       </c>
-      <c r="J34" t="str">
-        <v/>
+      <c r="J34">
+        <v>108</v>
       </c>
     </row>
     <row r="35">
@@ -1694,14 +1694,14 @@
       <c r="G35">
         <v>47</v>
       </c>
-      <c r="H35" t="str">
-        <v/>
+      <c r="H35">
+        <v>92</v>
       </c>
       <c r="I35">
         <v>83</v>
       </c>
-      <c r="J35" t="str">
-        <v/>
+      <c r="J35">
+        <v>128</v>
       </c>
     </row>
     <row r="36">
@@ -1726,14 +1726,14 @@
       <c r="G36">
         <v>101</v>
       </c>
-      <c r="H36" t="str">
-        <v/>
+      <c r="H36">
+        <v>121.4</v>
       </c>
       <c r="I36">
         <v>127</v>
       </c>
-      <c r="J36" t="str">
-        <v/>
+      <c r="J36">
+        <v>147.4</v>
       </c>
     </row>
     <row r="37">
@@ -1804,29 +1804,191 @@
       <c r="A39" t="str">
         <v>※ 선약현금가는 매장이 직접 입력 (공시지원금 + 공시현금가 공식은 매장지원금 차이에 따라 부정확)</v>
       </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
         <v>※ G·H·I·J 모두 매장이 직접 입력 (자동 계산 없음)</v>
       </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
         <v/>
       </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
         <v/>
       </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v/>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
         <v/>
       </c>
+      <c r="B43" t="str">
+        <v/>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
+        <v/>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
         <v/>
       </c>
     </row>

</xml_diff>